<commit_message>
GRS-0003 revision: B1/B3/B4/B8 content changes + ADR-0005/0006/0007
Acts on the golden-master review's content items (revise-before-ratify). Meridian
now: B=0.679 (group-weighted) P=0.380 L=0.484 -> V=0.511 (51.11); triad Economic
Established / Perceived Established / Defence Emerging.

- B1/ADR-0006: B is a GROUP-weighted mean so collinear scale metrics count once.
- B3: renamed TAKE_RATE_DURABILITY -> TAKE_RATE_LEVEL.
- B4: metrics and powers support NOT_APPLICABLE / NOT_ASSESSED with renormalisation.
- B8/ADR-0007: powers carry Benefit + Barrier (weaker gates, Helmer); N/A powers drop
  from P (0.271 -> 0.380); the triad is now DERIVED, ordinal out (ADR-0002).
- ADR-0005: B/P/L range comparability resolved by swing-weighted theta.

Workbook + regen script updated to match. ruff/pyright/pytest (72) + pre-commit green.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/golden-master.xlsx
+++ b/fixtures/golden-master.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -486,62 +486,83 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Subcomponents sheet (Basic/Developing/Advanced/Frontier, or blank + a State of</t>
+          <t>Subcomponents sheet (or set a State: NOT_APPLICABLE / NOT_ASSESSED) and q_m, L, B, P, V</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE / NOT_ASSESSED) and q_m, L, B, P and V recompute. Rating-gate bands are</t>
+          <t>recompute. B is a group-weighted mean (scale/unit-econ/momentum, ADR-0006); powers carry</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>rule-based (non-arithmetic, Methodology §5.2) and shown as computed values on Modules.</t>
+          <t>Benefit + Barrier and the weaker gates (Helmer); N/A powers drop from P. Gate bands</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>and the triad are rule-based/derived (computed values, regenerated by Python).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>DRAFT judgement calls for John to ratify: the subcomponent levels/evidence; the critical</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>flags; the uniform draft coefficients (α, δ, λ, θ, weights); the power-strength encoding</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>DRAFT judgement calls for John (GRS-0003 review): subcomponent levels/evidence; critical</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>(None=0, Emerging=0.4, Established=0.7, Wide=1.0); and the rating-gate rule. After an</t>
+          <t>flags; the N/A powers (Network Economies, Counter-Positioning); the draft coefficients</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>edit, save, then run scripts/regen_golden_master_json.py to refresh the JSON fixture.</t>
+          <t>(α, δ, λ, θ, group weights); the strength encoding (ADR-0004); the gate rule (ADR-0003);</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B/P range comparability (ADR-0005). Edit, save, then run</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Computed headline: B=0.679138  P=0.271429  L=0.483539  →  V=0.478586 (display 47.8586).</t>
+          <t>scripts/regen_golden_master_json.py to refresh the JSON fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Headline: B=0.67907  P=0.38  L=0.483539  →  V=0.511137 (display 51.1137).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Triad: Economic Established  ·  Perceived Established  ·  Defence Emerging.</t>
         </is>
       </c>
     </row>
@@ -2433,10 +2454,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2447,60 +2469,65 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
           <t>Raw</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Direction</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>x1</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>x2</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>x3</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>x4</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>y1</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>y2</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>y3</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>y4</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>n_k</t>
         </is>
@@ -2512,45 +2539,50 @@
           <t>AUA</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>1800000000</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>250000000</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>2000000000</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>20000000000</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.2</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0.5</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.8</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>1</v>
       </c>
-      <c r="M2">
-        <f>IF($B2&lt;=$E2,$I2,IF($B2&gt;=$H2,$L2,IF($B2&lt;=$F2,$I2+($B2-$E2)/($F2-$E2)*($J2-$I2),IF($B2&lt;=$G2,$J2+($B2-$F2)/($G2-$F2)*($K2-$J2),$K2+($B2-$G2)/($H2-$G2)*($L2-$K2))))))</f>
+      <c r="N2">
+        <f>IF(NOT(ISNUMBER($C2)),"",IF($C2&lt;=$F2,$J2,IF($C2&gt;=$I2,$M2,IF($C2&lt;=$G2,$J2+($C2-$F2)/($G2-$F2)*($K2-$J2),IF($C2&lt;=$H2,$K2+($C2-$G2)/($H2-$G2)*($L2-$K2),$L2+($C2-$H2)/($I2-$H2)*($M2-$L2))))))</f>
         <v/>
       </c>
     </row>
@@ -2560,45 +2592,50 @@
           <t>ACTIVE_CLIENTS</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>180000</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>25000</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>250000</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>2000000</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.2</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>0.5</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.8</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>1</v>
       </c>
-      <c r="M3">
-        <f>IF($B3&lt;=$E3,$I3,IF($B3&gt;=$H3,$L3,IF($B3&lt;=$F3,$I3+($B3-$E3)/($F3-$E3)*($J3-$I3),IF($B3&lt;=$G3,$J3+($B3-$F3)/($G3-$F3)*($K3-$J3),$K3+($B3-$G3)/($H3-$G3)*($L3-$K3))))))</f>
+      <c r="N3">
+        <f>IF(NOT(ISNUMBER($C3)),"",IF($C3&lt;=$F3,$J3,IF($C3&gt;=$I3,$M3,IF($C3&lt;=$G3,$J3+($C3-$F3)/($G3-$F3)*($K3-$J3),IF($C3&lt;=$H3,$K3+($C3-$G3)/($H3-$G3)*($L3-$K3),$L3+($C3-$H3)/($I3-$H3)*($M3-$L3))))))</f>
         <v/>
       </c>
     </row>
@@ -2608,45 +2645,50 @@
           <t>NET_REVENUE</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>85000000</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>10000000</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>100000000</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>1000000000</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>0.2</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>0.5</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>0.8</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>1</v>
       </c>
-      <c r="M4">
-        <f>IF($B4&lt;=$E4,$I4,IF($B4&gt;=$H4,$L4,IF($B4&lt;=$F4,$I4+($B4-$E4)/($F4-$E4)*($J4-$I4),IF($B4&lt;=$G4,$J4+($B4-$F4)/($G4-$F4)*($K4-$J4),$K4+($B4-$G4)/($H4-$G4)*($L4-$K4))))))</f>
+      <c r="N4">
+        <f>IF(NOT(ISNUMBER($C4)),"",IF($C4&lt;=$F4,$J4,IF($C4&gt;=$I4,$M4,IF($C4&lt;=$G4,$J4+($C4-$F4)/($G4-$F4)*($K4-$J4),IF($C4&lt;=$H4,$K4+($C4-$G4)/($H4-$G4)*($L4-$K4),$L4+($C4-$H4)/($I4-$H4)*($M4-$L4))))))</f>
         <v/>
       </c>
     </row>
@@ -2656,45 +2698,50 @@
           <t>REVENUE_PER_CLIENT</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>unit_economics</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>472</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>GBP_per_year</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>50</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>200</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>600</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>2000</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0.2</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>0.5</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>0.8</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>1</v>
       </c>
-      <c r="M5">
-        <f>IF($B5&lt;=$E5,$I5,IF($B5&gt;=$H5,$L5,IF($B5&lt;=$F5,$I5+($B5-$E5)/($F5-$E5)*($J5-$I5),IF($B5&lt;=$G5,$J5+($B5-$F5)/($G5-$F5)*($K5-$J5),$K5+($B5-$G5)/($H5-$G5)*($L5-$K5))))))</f>
+      <c r="N5">
+        <f>IF(NOT(ISNUMBER($C5)),"",IF($C5&lt;=$F5,$J5,IF($C5&gt;=$I5,$M5,IF($C5&lt;=$G5,$J5+($C5-$F5)/($G5-$F5)*($K5-$J5),IF($C5&lt;=$H5,$K5+($C5-$G5)/($H5-$G5)*($L5-$K5),$L5+($C5-$H5)/($I5-$H5)*($M5-$L5))))))</f>
         <v/>
       </c>
     </row>
@@ -2704,45 +2751,50 @@
           <t>GROSS_MARGIN</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>unit_economics</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>58</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>20</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>45</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>65</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>80</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>0.2</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>0.5</v>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>0.8</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>1</v>
       </c>
-      <c r="M6">
-        <f>IF($B6&lt;=$E6,$I6,IF($B6&gt;=$H6,$L6,IF($B6&lt;=$F6,$I6+($B6-$E6)/($F6-$E6)*($J6-$I6),IF($B6&lt;=$G6,$J6+($B6-$F6)/($G6-$F6)*($K6-$J6),$K6+($B6-$G6)/($H6-$G6)*($L6-$K6))))))</f>
+      <c r="N6">
+        <f>IF(NOT(ISNUMBER($C6)),"",IF($C6&lt;=$F6,$J6,IF($C6&gt;=$I6,$M6,IF($C6&lt;=$G6,$J6+($C6-$F6)/($G6-$F6)*($K6-$J6),IF($C6&lt;=$H6,$K6+($C6-$G6)/($H6-$G6)*($L6-$K6),$L6+($C6-$H6)/($I6-$H6)*($M6-$L6))))))</f>
         <v/>
       </c>
     </row>
@@ -2752,189 +2804,209 @@
           <t>COST_TO_SERVE</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>unit_economics</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>140</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>GBP_per_year</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>lower_is_better</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>40</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>100</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>200</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>400</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>0.8</v>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>0.5</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>0.2</v>
       </c>
-      <c r="M7">
-        <f>IF($B7&lt;=$E7,$I7,IF($B7&gt;=$H7,$L7,IF($B7&lt;=$F7,$I7+($B7-$E7)/($F7-$E7)*($J7-$I7),IF($B7&lt;=$G7,$J7+($B7-$F7)/($G7-$F7)*($K7-$J7),$K7+($B7-$G7)/($H7-$G7)*($L7-$K7))))))</f>
+      <c r="N7">
+        <f>IF(NOT(ISNUMBER($C7)),"",IF($C7&lt;=$F7,$J7,IF($C7&gt;=$I7,$M7,IF($C7&lt;=$G7,$J7+($C7-$F7)/($G7-$F7)*($K7-$J7),IF($C7&lt;=$H7,$K7+($C7-$G7)/($H7-$G7)*($L7-$K7),$L7+($C7-$H7)/($I7-$H7)*($M7-$L7))))))</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>NET_REVENUE_RETENTION</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>104</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>percent</t>
-        </is>
+          <t>TAKE_RATE_LEVEL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>unit_economics</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>22</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>bps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>80</v>
-      </c>
       <c r="F8" t="n">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="G8" t="n">
-        <v>110</v>
+        <v>15</v>
       </c>
       <c r="H8" t="n">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="I8" t="n">
+        <v>60</v>
+      </c>
+      <c r="J8" t="n">
         <v>0.2</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>0.5</v>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>0.8</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>1</v>
       </c>
-      <c r="M8">
-        <f>IF($B8&lt;=$E8,$I8,IF($B8&gt;=$H8,$L8,IF($B8&lt;=$F8,$I8+($B8-$E8)/($F8-$E8)*($J8-$I8),IF($B8&lt;=$G8,$J8+($B8-$F8)/($G8-$F8)*($K8-$J8),$K8+($B8-$G8)/($H8-$G8)*($L8-$K8))))))</f>
+      <c r="N8">
+        <f>IF(NOT(ISNUMBER($C8)),"",IF($C8&lt;=$F8,$J8,IF($C8&gt;=$I8,$M8,IF($C8&lt;=$G8,$J8+($C8-$F8)/($G8-$F8)*($K8-$J8),IF($C8&lt;=$H8,$K8+($C8-$G8)/($H8-$G8)*($L8-$K8),$L8+($C8-$H8)/($I8-$H8)*($M8-$L8))))))</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLIENT_GROWTH_RATE</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>14</v>
-      </c>
-      <c r="C9" t="inlineStr">
+          <t>NET_REVENUE_RETENTION</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>momentum</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>104</v>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>percent</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
       <c r="F9" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="G9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="H9" t="n">
-        <v>50</v>
+        <v>110</v>
       </c>
       <c r="I9" t="n">
+        <v>130</v>
+      </c>
+      <c r="J9" t="n">
         <v>0.2</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>0.5</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>0.8</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>1</v>
       </c>
-      <c r="M9">
-        <f>IF($B9&lt;=$E9,$I9,IF($B9&gt;=$H9,$L9,IF($B9&lt;=$F9,$I9+($B9-$E9)/($F9-$E9)*($J9-$I9),IF($B9&lt;=$G9,$J9+($B9-$F9)/($G9-$F9)*($K9-$J9),$K9+($B9-$G9)/($H9-$G9)*($L9-$K9))))))</f>
+      <c r="N9">
+        <f>IF(NOT(ISNUMBER($C9)),"",IF($C9&lt;=$F9,$J9,IF($C9&gt;=$I9,$M9,IF($C9&lt;=$G9,$J9+($C9-$F9)/($G9-$F9)*($K9-$J9),IF($C9&lt;=$H9,$K9+($C9-$G9)/($H9-$G9)*($L9-$K9),$L9+($C9-$H9)/($I9-$H9)*($M9-$L9))))))</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TAKE_RATE_DURABILITY</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>22</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>bps</t>
-        </is>
+          <t>CLIENT_GROWTH_RATE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>momentum</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>14</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>higher_is_better</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>5</v>
-      </c>
       <c r="F10" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H10" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="I10" t="n">
+        <v>50</v>
+      </c>
+      <c r="J10" t="n">
         <v>0.2</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>0.5</v>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>0.8</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>1</v>
       </c>
-      <c r="M10">
-        <f>IF($B10&lt;=$E10,$I10,IF($B10&gt;=$H10,$L10,IF($B10&lt;=$F10,$I10+($B10-$E10)/($F10-$E10)*($J10-$I10),IF($B10&lt;=$G10,$J10+($B10-$F10)/($G10-$F10)*($K10-$J10),$K10+($B10-$G10)/($H10-$G10)*($L10-$K10))))))</f>
+      <c r="N10">
+        <f>IF(NOT(ISNUMBER($C10)),"",IF($C10&lt;=$F10,$J10,IF($C10&gt;=$I10,$M10,IF($C10&lt;=$G10,$J10+($C10-$F10)/($G10-$F10)*($K10-$J10),IF($C10&lt;=$H10,$K10+($C10-$G10)/($H10-$G10)*($L10-$K10),$L10+($C10-$H10)/($I10-$H10)*($M10-$L10))))))</f>
         <v/>
       </c>
     </row>
@@ -2944,56 +3016,101 @@
           <t>CAC_PAYBACK_MONTHS</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>momentum</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>18</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>months</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>lower_is_better</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>6</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>12</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>24</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>48</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>0.8</v>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>0.5</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>0.2</v>
       </c>
-      <c r="M11">
-        <f>IF($B11&lt;=$E11,$I11,IF($B11&gt;=$H11,$L11,IF($B11&lt;=$F11,$I11+($B11-$E11)/($F11-$E11)*($J11-$I11),IF($B11&lt;=$G11,$J11+($B11-$F11)/($G11-$F11)*($K11-$J11),$K11+($B11-$G11)/($H11-$G11)*($L11-$K11))))))</f>
+      <c r="N11">
+        <f>IF(NOT(ISNUMBER($C11)),"",IF($C11&lt;=$F11,$J11,IF($C11&gt;=$I11,$M11,IF($C11&lt;=$G11,$J11+($C11-$F11)/($G11-$F11)*($K11-$J11),IF($C11&lt;=$H11,$K11+($C11-$G11)/($H11-$G11)*($L11-$K11),$L11+($C11-$H11)/($I11-$H11)*($M11-$L11))))))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Group means (group-weighted B, ADR-0006):</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+      <c r="N13">
+        <f>AVERAGEIF($B$2:$B$11,"scale",$N$2:$N$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>unit_economics</t>
+        </is>
+      </c>
+      <c r="N14">
+        <f>AVERAGEIF($B$2:$B$11,"unit_economics",$N$2:$N$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>momentum</t>
+        </is>
+      </c>
+      <c r="N15">
+        <f>AVERAGEIF($B$2:$B$11,"momentum",$N$2:$N$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="M16" t="inlineStr">
         <is>
           <t>B =</t>
         </is>
       </c>
-      <c r="M12" s="4">
-        <f>AVERAGE($M$2:$M$11)</f>
+      <c r="N16" s="4">
+        <f>AVERAGE($N$13,$N$14,$N$15)</f>
         <v/>
       </c>
     </row>
@@ -3008,10 +3125,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3022,12 +3140,27 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Strength</t>
+          <t>Benefit</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Barrier</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Strength (weaker)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
           <t>Value</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>State</t>
         </is>
       </c>
     </row>
@@ -3042,8 +3175,17 @@
           <t>Emerging</t>
         </is>
       </c>
-      <c r="C2">
-        <f>IF($B2="None",0,IF($B2="Emerging",0.4,IF($B2="Established",0.7,IF($B2="Wide",1,""))))</f>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="D2">
+        <f>IF((IF($B2="None",0,IF($B2="Emerging",1,IF($B2="Established",2,3))))&lt;=(IF($C2="None",0,IF($C2="Emerging",1,IF($C2="Established",2,3)))),$B2,$C2)</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>IF($D2="","",IF($D2="None",0,IF($D2="Emerging",0.4,IF($D2="Established",0.7,IF($D2="Wide",1,"")))))</f>
         <v/>
       </c>
     </row>
@@ -3053,14 +3195,10 @@
           <t>NETWORK_ECONOMIES</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C3">
-        <f>IF($B3="None",0,IF($B3="Emerging",0.4,IF($B3="Established",0.7,IF($B3="Wide",1,""))))</f>
-        <v/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NOT_APPLICABLE</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3069,14 +3207,10 @@
           <t>COUNTER_POSITIONING</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="C4">
-        <f>IF($B4="None",0,IF($B4="Emerging",0.4,IF($B4="Established",0.7,IF($B4="Wide",1,""))))</f>
-        <v/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NOT_APPLICABLE</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3090,8 +3224,17 @@
           <t>Established</t>
         </is>
       </c>
-      <c r="C5">
-        <f>IF($B5="None",0,IF($B5="Emerging",0.4,IF($B5="Established",0.7,IF($B5="Wide",1,""))))</f>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="D5">
+        <f>IF((IF($B5="None",0,IF($B5="Emerging",1,IF($B5="Established",2,3))))&lt;=(IF($C5="None",0,IF($C5="Emerging",1,IF($C5="Established",2,3)))),$B5,$C5)</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>IF($D5="","",IF($D5="None",0,IF($D5="Emerging",0.4,IF($D5="Established",0.7,IF($D5="Wide",1,"")))))</f>
         <v/>
       </c>
     </row>
@@ -3106,8 +3249,17 @@
           <t>Emerging</t>
         </is>
       </c>
-      <c r="C6">
-        <f>IF($B6="None",0,IF($B6="Emerging",0.4,IF($B6="Established",0.7,IF($B6="Wide",1,""))))</f>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="D6">
+        <f>IF((IF($B6="None",0,IF($B6="Emerging",1,IF($B6="Established",2,3))))&lt;=(IF($C6="None",0,IF($C6="Emerging",1,IF($C6="Established",2,3)))),$B6,$C6)</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>IF($D6="","",IF($D6="None",0,IF($D6="Emerging",0.4,IF($D6="Established",0.7,IF($D6="Wide",1,"")))))</f>
         <v/>
       </c>
     </row>
@@ -3122,8 +3274,17 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C7">
-        <f>IF($B7="None",0,IF($B7="Emerging",0.4,IF($B7="Established",0.7,IF($B7="Wide",1,""))))</f>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D7">
+        <f>IF((IF($B7="None",0,IF($B7="Emerging",1,IF($B7="Established",2,3))))&lt;=(IF($C7="None",0,IF($C7="Emerging",1,IF($C7="Established",2,3)))),$B7,$C7)</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>IF($D7="","",IF($D7="None",0,IF($D7="Emerging",0.4,IF($D7="Established",0.7,IF($D7="Wide",1,"")))))</f>
         <v/>
       </c>
     </row>
@@ -3138,19 +3299,28 @@
           <t>Emerging</t>
         </is>
       </c>
-      <c r="C8">
-        <f>IF($B8="None",0,IF($B8="Emerging",0.4,IF($B8="Established",0.7,IF($B8="Wide",1,""))))</f>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
+      </c>
+      <c r="D8">
+        <f>IF((IF($B8="None",0,IF($B8="Emerging",1,IF($B8="Established",2,3))))&lt;=(IF($C8="None",0,IF($C8="Emerging",1,IF($C8="Established",2,3)))),$B8,$C8)</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IF($D8="","",IF($D8="None",0,IF($D8="Emerging",0.4,IF($D8="Established",0.7,IF($D8="Wide",1,"")))))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>P =</t>
         </is>
       </c>
-      <c r="C9" s="4">
-        <f>AVERAGE($C$2:$C$8)</f>
+      <c r="E9" s="4">
+        <f>AVERAGE($E$2:$E$8)</f>
         <v/>
       </c>
     </row>
@@ -3165,10 +3335,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
@@ -3247,7 +3417,7 @@
         </is>
       </c>
       <c r="C7">
-        <f>Business!$M$12</f>
+        <f>Business!$N$16</f>
         <v/>
       </c>
     </row>
@@ -3258,7 +3428,7 @@
         </is>
       </c>
       <c r="C8">
-        <f>Powers!$C$9</f>
+        <f>Powers!$E$9</f>
         <v/>
       </c>
     </row>
@@ -3312,6 +3482,52 @@
       <c r="C13">
         <f>$C12*100</f>
         <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>— Platform Power Triad (ordinal, ADR-0007) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Economic Value</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Perceived Value</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Defence Value</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Emerging</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
GRS-0005 precursor: golden master uses contract enum VALUES for states
Audit follow-up from GRS-0004. The fixture stored non-score states as the enum
NAMES (NOT_APPLICABLE); the engine emits the contract enum VALUES
(Not Applicable / Not Assessed). Align on the single contract vocabulary (D8) so
Monte Carlo reads a contract-vocabulary oracle:

- build_golden_master.py binds NOT_APPLICABLE/NOT_ASSESSED to
  NonScoreState.*.value; regenerate the fixture (only the 3 subcomponent state
  strings change — every ratified number is byte-stable, V=0.478565).
- Delete the _state_value alias in the golden-master test; states compare
  directly now.
- Update the GRS-0003 fixture/gate tests to the contract vocabulary.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/golden-master.xlsx
+++ b/fixtures/golden-master.xlsx
@@ -1213,7 +1213,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>Not Assessed</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
-          <t>NOT_ASSESSED</t>
+          <t>Not Assessed</t>
         </is>
       </c>
     </row>

</xml_diff>